<commit_message>
Act generator: robust GTD number pick, content-based XLSX detection, house-style dates
Pick the declaration number from the filename or the most frequent match
(declarations reference other DTs in graph 44). Detect fact/order XLSX by
headers, skip duplicate PDFs, write signature dates as '"14" сентября 2026г.'.
Case CP-1-2026 now built from the real GTD and fact packing list.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPDW65Tn1skVQugzZKtH
</commit_message>
<xml_diff>
--- a/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
+++ b/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
@@ -4526,7 +4526,7 @@
     <row r="9" ht="18.75" customHeight="1" s="47">
       <c r="B9" s="137" t="inlineStr">
         <is>
-          <t xml:space="preserve">от </t>
+          <t>от 14.09.2026 г.</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,9 @@
           <t>Дата выезда продукции (товара) из г. Стамбул:</t>
         </is>
       </c>
-      <c r="G15" s="310" t="n"/>
+      <c r="G15" s="316" t="n">
+        <v>46231</v>
+      </c>
       <c r="H15" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve"> г.</t>
@@ -4679,7 +4681,9 @@
           <t>Дата поступления продукции (товара) на склад:</t>
         </is>
       </c>
-      <c r="G17" s="310" t="n"/>
+      <c r="G17" s="316" t="n">
+        <v>46272</v>
+      </c>
       <c r="H17" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve"> г.</t>
@@ -6515,7 +6519,7 @@
       </c>
       <c r="F76" s="315" t="inlineStr">
         <is>
-          <t>"  "                 2026г.</t>
+          <t>"14" сентября 2026г.</t>
         </is>
       </c>
       <c r="G76" s="50" t="n"/>
@@ -6620,7 +6624,7 @@
       </c>
       <c r="F79" s="315" t="inlineStr">
         <is>
-          <t>"  "                 2026г.</t>
+          <t>"14" сентября 2026г.</t>
         </is>
       </c>
       <c r="G79" s="50" t="n"/>
@@ -6717,7 +6721,7 @@
       </c>
       <c r="F82" s="315" t="inlineStr">
         <is>
-          <t>"  "                 2026г.</t>
+          <t>"14" сентября 2026г.</t>
         </is>
       </c>
       <c r="G82" s="50" t="n"/>

</xml_diff>

<commit_message>
Act generator: 1C receipt for stage 3, article normalization, invoices 1043/1165 from PDF
Stage 3 compares invoice vs 1C line totals (unit-of-measure differences such as
2 m duct pieces are noted, not flagged). Article codes normalized (spaces),
split 1C lines aggregated. Case CP-1-2026 now has all KVT invoices but 1276.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPDW65Tn1skVQugzZKtH
</commit_message>
<xml_diff>
--- a/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
+++ b/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
@@ -5511,7 +5511,11 @@
       <c r="M41" s="331" t="n"/>
       <c r="N41" s="331" t="n"/>
       <c r="O41" s="330" t="n"/>
-      <c r="P41" s="348" t="n"/>
+      <c r="P41" s="348" t="inlineStr">
+        <is>
+          <t>Сверено с документом 1С «Приобретение товаров № КА-358 от 24 августа 2026 г.». Разная ед. изм. без расхождения по сумме: 17 поз. (CWD) — цена в 1С ×2.0, кол-во соответственно меньше</t>
+        </is>
+      </c>
       <c r="Q41" s="320" t="n"/>
       <c r="R41" s="320" t="n"/>
       <c r="S41" s="319" t="n"/>

</xml_diff>

<commit_message>
Act generator: printable PDF form, row visibility matching the template
render.py turns the generated act into a one-page A4 landscape PDF/PNG that
mirrors the company's printed standard (merged cells, borders, fonts, evaluated
formulas, hidden rows skipped). akt.py now unhides/hides stage 2 and 4 rows to
the actual number of discrepancies, formats packing summary in Russian style,
and sets fit-to-page print setup.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbPDW65Tn1skVQugzZKtH
</commit_message>
<xml_diff>
--- a/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
+++ b/akt-priemki/cases/CP-1-2026/Акт приёмки №1 (СР отгрузка 1 в 26).xlsx
@@ -2353,7 +2353,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="372">
+  <cellXfs count="373">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3371,6 +3371,9 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="35" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4566,7 +4569,7 @@
       <c r="A12" s="49" t="n"/>
       <c r="B12" s="308" t="inlineStr">
         <is>
-          <t>Упаковочный лист (количество мест,  вес, объем) 0 коробок, 19 паллет, 54.13 м³, вес брутто - 7506 кг, вес нетто - 7296 кг.</t>
+          <t>Упаковочный лист (количество мест,  вес, объем) 19 паллет, 54,13 м³, вес брутто - 7 506 кг, вес нетто - 7 296 кг.</t>
         </is>
       </c>
       <c r="U12" s="143" t="n"/>
@@ -5139,7 +5142,7 @@
       <c r="U30" s="328" t="n"/>
       <c r="V30" s="49" t="n"/>
     </row>
-    <row r="31" hidden="1" ht="15.75" customHeight="1" s="47">
+    <row r="31" ht="15.75" customHeight="1" s="47">
       <c r="A31" s="49" t="n"/>
       <c r="B31" s="336" t="n"/>
       <c r="C31" s="337" t="n"/>
@@ -5183,7 +5186,7 @@
       <c r="U31" s="328" t="n"/>
       <c r="V31" s="49" t="n"/>
     </row>
-    <row r="32" hidden="1" ht="15.75" customHeight="1" s="47">
+    <row r="32" ht="15.75" customHeight="1" s="47">
       <c r="A32" s="49" t="n"/>
       <c r="B32" s="336" t="n"/>
       <c r="C32" s="337" t="n"/>
@@ -5227,7 +5230,7 @@
       <c r="U32" s="328" t="n"/>
       <c r="V32" s="49" t="n"/>
     </row>
-    <row r="33" hidden="1" ht="18.75" customHeight="1" s="47">
+    <row r="33" ht="18.75" customHeight="1" s="47">
       <c r="A33" s="49" t="n"/>
       <c r="B33" s="336" t="n"/>
       <c r="C33" s="337" t="n"/>
@@ -5271,7 +5274,7 @@
       <c r="U33" s="328" t="n"/>
       <c r="V33" s="49" t="n"/>
     </row>
-    <row r="34" hidden="1" ht="16.5" customHeight="1" s="47">
+    <row r="34" ht="16.5" customHeight="1" s="47">
       <c r="A34" s="49" t="n"/>
       <c r="B34" s="336" t="n"/>
       <c r="C34" s="337" t="n"/>
@@ -5315,7 +5318,7 @@
       <c r="U34" s="328" t="n"/>
       <c r="V34" s="49" t="n"/>
     </row>
-    <row r="35" hidden="1" ht="15.75" customHeight="1" s="47">
+    <row r="35" ht="15.75" customHeight="1" s="47">
       <c r="A35" s="49" t="n"/>
       <c r="B35" s="336" t="n"/>
       <c r="C35" s="337" t="n"/>
@@ -5562,7 +5565,7 @@
       </c>
       <c r="U42" s="319" t="n"/>
     </row>
-    <row r="43" ht="24.75" customHeight="1" s="47" thickBot="1">
+    <row r="43" hidden="1" ht="24.75" customHeight="1" s="47" thickBot="1">
       <c r="B43" s="336" t="n"/>
       <c r="C43" s="337" t="n"/>
       <c r="D43" s="328" t="n"/>
@@ -6683,7 +6686,7 @@
         </is>
       </c>
       <c r="T80" s="362" t="n"/>
-      <c r="U80" s="40">
+      <c r="U80" s="368">
         <f>U79/U78</f>
         <v/>
       </c>
@@ -7010,7 +7013,7 @@
     <mergeCell ref="E27:K27"/>
   </mergeCells>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.3543307086614174" bottom="0.1574803149606299" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="50" fitToHeight="2"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="50" fitToHeight="1" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="65" min="0" max="20" man="1"/>
   </rowBreaks>
@@ -7077,7 +7080,7 @@
           <t>1$ доллар</t>
         </is>
       </c>
-      <c r="B4" s="368">
+      <c r="B4" s="369">
         <f>'СР отгрузка 1 в 26'!U78</f>
         <v/>
       </c>
@@ -7089,7 +7092,7 @@
           <t>1евро</t>
         </is>
       </c>
-      <c r="B5" s="369">
+      <c r="B5" s="370">
         <f>'СР отгрузка 1 в 26'!U79</f>
         <v/>
       </c>
@@ -7126,7 +7129,7 @@
       <c r="O7" s="35" t="n"/>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="47" thickBot="1">
-      <c r="A8" s="370" t="inlineStr">
+      <c r="A8" s="371" t="inlineStr">
         <is>
           <t>Затраты на доставку и ТО</t>
         </is>
@@ -7340,7 +7343,7 @@
           <t>EMAS</t>
         </is>
       </c>
-      <c r="B12" s="371">
+      <c r="B12" s="372">
         <f>'СР отгрузка 1 в 26'!F19</f>
         <v/>
       </c>

</xml_diff>